<commit_message>
after 2026-3 commissioning beamtime
BLOP work
+ predict dcm.roll based on early results from BLOP session and use it
  in change_edge()
+ scan roll option in change edge command
+ poll Tiled carefully to deal with network slowdown from Sep 22 to
  Oct 1

goniometer and bluesky
+ update KNOWN_ATTENUATION with better numbers from both Jean and
  Donald
+ improve plotting with mythen, start plotting with eiger
+ plot against "ic0" for gonio profile
+ very crude stab at capturing egu in plot ... needs imrpovement
+ make XRR live plotting work correctly
+ poll Tiled carefully to deal with network slowdown from Sep 22 to
  Oct 1
+ quick-n-dirty of plot of completed xrr scans from bsui command line
+ identify catalog.is_sql and .uri when consumers start
+ write usable Mtalab out files for XRR
+ use .read() consistently throughout when access data from Tiled
</commit_message>
<xml_diff>
--- a/startup/lookup_table/Modes.xlsx
+++ b/startup/lookup_table/Modes.xlsx
@@ -11902,7 +11902,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ66"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.04"/>
@@ -13979,7 +13979,7 @@
         <v>2679</v>
       </c>
       <c r="T40" s="33" t="n">
-        <v>-0.065</v>
+        <v>-1.249</v>
       </c>
       <c r="U40" s="0" t="n">
         <v>1252</v>
@@ -14033,7 +14033,7 @@
         <v>-10199</v>
       </c>
       <c r="T41" s="33" t="n">
-        <v>0.471</v>
+        <v>-1.345</v>
       </c>
       <c r="U41" s="0" t="n">
         <v>-8786</v>
@@ -14895,7 +14895,7 @@
         <v>141529</v>
       </c>
       <c r="T54" s="57" t="n">
-        <v>58.444</v>
+        <v>58.6936</v>
       </c>
       <c r="U54" s="28" t="n">
         <v>497477</v>
@@ -15049,7 +15049,7 @@
       <c r="R56" s="26"/>
       <c r="S56" s="26"/>
       <c r="T56" s="55" t="n">
-        <v>141.1</v>
+        <v>140.1</v>
       </c>
       <c r="U56" s="25" t="n">
         <v>10530029</v>
@@ -15162,7 +15162,7 @@
         <v>4479629</v>
       </c>
       <c r="T58" s="55" t="n">
-        <v>143.4</v>
+        <v>142.4</v>
       </c>
       <c r="U58" s="28" t="n">
         <v>6889105</v>
@@ -17181,7 +17181,7 @@
       </c>
       <c r="F30" s="110" t="n">
         <f aca="false">'Modes A-F'!T54</f>
-        <v>58.444</v>
+        <v>58.6936</v>
       </c>
       <c r="G30" s="0"/>
       <c r="H30" s="0"/>
@@ -17226,7 +17226,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:K7"/>
-  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
@@ -17405,7 +17405,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.96"/>
@@ -17976,7 +17976,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CX484"/>
-  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="2" style="0" width="11.96"/>
@@ -24043,7 +24043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2383"/>
-  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.14"/>

</xml_diff>